<commit_message>
Actualizo README de Prueba 1 y subo Excel mejorado
</commit_message>
<xml_diff>
--- a/Prueba-01-Analisis-Datos/solucion.xlsx
+++ b/Prueba-01-Analisis-Datos/solucion.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="2"/>
+    <workbookView xWindow="600" yWindow="460" windowWidth="28200" windowHeight="17540" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Material de apoyo - Prueba " sheetId="7" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1728" uniqueCount="686">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1715" uniqueCount="673">
   <si>
     <t>Fecha</t>
   </si>
@@ -1956,21 +1956,6 @@
     <t>Tabla 2: Productos (ID_Producto, Nombre, Categoría, Precio_Unitario)</t>
   </si>
   <si>
-    <t>¿Cómo relacionarías estas tablas en Power Pivot?</t>
-  </si>
-  <si>
-    <t>El problema es que en Ventas solo guardas el código del producto (P001, P002...), no el nombre ni el precio. Power Pivot necesita saber cómo unirlas.</t>
-  </si>
-  <si>
-    <t>El proceso en 3 pasos simples</t>
-  </si>
-  <si>
-    <t>¿Qué logras con eso?</t>
-  </si>
-  <si>
-    <t>A partir de ese momento puedes crear medidas que usen datos de las dos tablas al mismo tiempo, como calcular el margen de ganancia multiplicando la cantidad vendida (que está en Ventas) por el precio (que está en Productos).</t>
-  </si>
-  <si>
     <t>Margen de Ganancia</t>
   </si>
   <si>
@@ -2080,180 +2065,6 @@
   </si>
   <si>
     <t>Quitar Duplicados (Datos)</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Ventas </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">— cada vez que alguien compró algo </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Productos</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> — la ficha de cada producto </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>1. Cargar las tablas</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Seleccionas tu tabla de Ventas → clic en </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"Agregar al modelo de datos"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Repites con Productos.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>2. Ir al diagrama</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Dentro de Power Pivot, cambias a </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>"Vista de diagrama"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> y ves las dos tablas como cajitas.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>3. Arrastrar el campo en común</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Tomas ID_Producto de la tabla Ventas y lo arrastras encima de ID_Producto de Productos. Se dibuja una línea entre las dos tablas. Eso es todo.</t>
-    </r>
-  </si>
-  <si>
-    <t>Que Power Pivot sepa que cuando ve P001 en Ventas, debe ir a buscar el nombre, la categoría y el precio a la tabla Productos. Sin necesidad de escribir ningún VLOOKUP.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Medida DAX </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(referencia, ya que mi Mac no tiene Power Pivot):</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Margen de Ganancia =</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> DIVIDE(SUM(Ventas[Monto]) - SUM(Ventas[Cantidad] * Productos[Costo_Unitario]), SUM(Ventas[Monto]))</t>
-    </r>
   </si>
 </sst>
 </file>
@@ -2555,7 +2366,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="8">
+  <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -2564,6 +2375,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -2739,13 +2552,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="8">
+  <cellStyles count="10">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hipervínculo" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hipervínculo" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="8" builtinId="8" hidden="1"/>
     <cellStyle name="Hipervínculo visitado" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Hipervínculo visitado" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Hipervínculo visitado" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="9" builtinId="9" hidden="1"/>
     <cellStyle name="Moneda [0]" xfId="7" builtinId="7"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -3175,11 +2990,11 @@
         </c:hiLowLines>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="2128685584"/>
-        <c:axId val="2128691632"/>
+        <c:axId val="2110981280"/>
+        <c:axId val="2110987328"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2128685584"/>
+        <c:axId val="2110981280"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3254,7 +3069,7 @@
             <a:endParaRPr lang="es-ES_tradnl"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2128691632"/>
+        <c:crossAx val="2110987328"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3262,7 +3077,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2128691632"/>
+        <c:axId val="2110987328"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3345,7 +3160,7 @@
             <a:endParaRPr lang="es-ES_tradnl"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2128685584"/>
+        <c:crossAx val="2110981280"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
         <c:majorUnit val="4000.0"/>
@@ -3449,6 +3264,346 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6540500" cy="7581900"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="CuadroTexto 1"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10490200" y="533400"/>
+          <a:ext cx="6540500" cy="7581900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1800" b="1"/>
+            <a:t>¿Cómo relacionarías estas tablas en Power Pivot?</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t/>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+          </a:br>
+          <a:endParaRPr lang="es-ES_tradnl" sz="1400"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>Ventas</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t> — cada vez que alguien compró algo.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>Productos</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t> — la ficha de cada producto.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+          </a:br>
+          <a:endParaRPr lang="es-ES_tradnl" sz="1400"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>El problema es que en </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>Ventas</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t> solo guardas el código del producto (P001, P002...), no el nombre ni el precio. Power Pivot necesita saber cómo unirlas.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+          </a:br>
+          <a:endParaRPr lang="es-ES_tradnl" sz="1400"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>El proceso en 3 pasos simples</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>1. Cargar las tablas</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-ES_tradnl" sz="1400"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>Seleccionas tu tabla de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>Ventas</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t> → clic en </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>"Agregar al modelo de datos"</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+          </a:br>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>Repites el proceso con </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>Productos</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+          </a:br>
+          <a:endParaRPr lang="es-ES_tradnl" sz="1400"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>2. Ir al diagrama</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-ES_tradnl" sz="1400"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>Dentro de Power Pivot, cambias a </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>"Vista de diagrama"</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t> y ves las dos tablas como cajitas.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+          </a:br>
+          <a:endParaRPr lang="es-ES_tradnl" sz="1400"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>3. Arrastrar el campo en común</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-ES_tradnl" sz="1400"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>Tomas </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>ID_Producto</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t> de la tabla </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>Ventas</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t> y lo arrastras encima de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>ID_Producto</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t> de </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>Productos</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>Se dibuja una línea entre las dos tablas. Eso es todo.</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+          </a:br>
+          <a:endParaRPr lang="es-ES_tradnl" sz="1400"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>¿Qué logras con eso?</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>Power Pivot sabe que, cuando ve </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>P001</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t> en Ventas, debe ir a buscar el nombre, la categoría y el precio a la tabla </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>Productos</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>, sin necesidad de escribir ningún </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>VLOOKUP</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>A partir de ese momento puedes crear medidas que usen datos de las dos tablas al mismo tiempo, como calcular el margen de ganancia multiplicando la cantidad vendida (que está en </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>Ventas</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>) por el precio (que está en </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>Productos</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>).</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+          </a:br>
+          <a:endParaRPr lang="es-ES_tradnl" sz="1400"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" b="1"/>
+            <a:t>Medida DAX</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400" i="1"/>
+            <a:t>Referencia, ya que mi Mac no tiene Power Pivot:</a:t>
+          </a:r>
+          <a:endParaRPr lang="es-ES_tradnl" sz="1400"/>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="es-ES_tradnl" sz="1400"/>
+            <a:t>Margen de Ganancia = DIVIDE( SUM(Ventas[Monto]) - SUM(Ventas[Cantidad] * Productos[Costo_Unitario]), SUM(Ventas[Monto]) )  </a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
@@ -3537,10 +3692,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="Tabla7" displayName="Tabla7" ref="B13:E17" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
   <autoFilter ref="B13:E17"/>
   <tableColumns count="4">
-    <tableColumn id="1" name="#" dataDxfId="3"/>
-    <tableColumn id="2" name="Problema Detectado" dataDxfId="2"/>
-    <tableColumn id="3" name="Técnica de Excel" dataDxfId="1"/>
-    <tableColumn id="4" name="Resultado" dataDxfId="0"/>
+    <tableColumn id="1" name="#" dataDxfId="1"/>
+    <tableColumn id="2" name="Problema Detectado" dataDxfId="0"/>
+    <tableColumn id="3" name="Técnica de Excel" dataDxfId="3"/>
+    <tableColumn id="4" name="Resultado" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -10860,97 +11015,97 @@
     <row r="1" spans="2:5" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:5" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B2" s="10" t="s">
-        <v>676</v>
+        <v>671</v>
       </c>
     </row>
     <row r="3" spans="2:5" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B4" s="11" t="s">
-        <v>642</v>
+        <v>637</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>644</v>
+        <v>639</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>646</v>
+        <v>641</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>645</v>
+        <v>640</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="57" x14ac:dyDescent="0.2">
       <c r="B5" s="12" t="s">
-        <v>647</v>
+        <v>642</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>648</v>
+        <v>643</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>649</v>
+        <v>644</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>643</v>
+        <v>638</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="38" x14ac:dyDescent="0.2">
       <c r="B6" s="12" t="s">
-        <v>650</v>
+        <v>645</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>651</v>
+        <v>646</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>652</v>
+        <v>647</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>653</v>
+        <v>648</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="57" x14ac:dyDescent="0.2">
       <c r="B7" s="12" t="s">
-        <v>654</v>
+        <v>649</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>655</v>
+        <v>650</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>656</v>
+        <v>651</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>653</v>
+        <v>648</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="38" x14ac:dyDescent="0.2">
       <c r="B8" s="12" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>658</v>
+        <v>653</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>659</v>
+        <v>654</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>660</v>
+        <v>655</v>
       </c>
     </row>
     <row r="9" spans="2:5" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="10" spans="2:5" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="11" spans="2:5" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B11" s="10" t="s">
-        <v>661</v>
+        <v>656</v>
       </c>
     </row>
     <row r="12" spans="2:5" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
     <row r="13" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B13" s="15" t="s">
-        <v>662</v>
+        <v>657</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>663</v>
+        <v>658</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>664</v>
+        <v>659</v>
       </c>
       <c r="E13" s="15" t="s">
         <v>456</v>
@@ -10961,13 +11116,13 @@
         <v>1</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>665</v>
+        <v>660</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>666</v>
+        <v>661</v>
       </c>
     </row>
     <row r="15" spans="2:5" ht="38" x14ac:dyDescent="0.2">
@@ -10975,13 +11130,13 @@
         <v>2</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>667</v>
+        <v>662</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>668</v>
+        <v>663</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>669</v>
+        <v>664</v>
       </c>
     </row>
     <row r="16" spans="2:5" ht="38" x14ac:dyDescent="0.2">
@@ -10989,13 +11144,13 @@
         <v>3</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>670</v>
+        <v>665</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>671</v>
+        <v>666</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>672</v>
+        <v>667</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="38" x14ac:dyDescent="0.2">
@@ -11003,13 +11158,13 @@
         <v>4</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>673</v>
+        <v>668</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>674</v>
+        <v>669</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>675</v>
+        <v>670</v>
       </c>
     </row>
     <row r="18" spans="2:5" s="9" customFormat="1" x14ac:dyDescent="0.2"/>
@@ -14252,7 +14407,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:G65"/>
+  <dimension ref="B2:G38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="53"/>
@@ -14262,7 +14417,9 @@
     <col min="5" max="5" width="15.1640625" style="53" customWidth="1"/>
     <col min="6" max="6" width="18.6640625" style="53" customWidth="1"/>
     <col min="7" max="7" width="22.5" style="60" customWidth="1"/>
-    <col min="8" max="16384" width="10.83203125" style="53"/>
+    <col min="8" max="8" width="10.83203125" style="53"/>
+    <col min="9" max="14" width="10.83203125" style="53" customWidth="1"/>
+    <col min="15" max="16384" width="10.83203125" style="53"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" s="49" customFormat="1" x14ac:dyDescent="0.25">
@@ -14288,7 +14445,7 @@
         <v>2</v>
       </c>
       <c r="G4" s="52" t="s">
-        <v>641</v>
+        <v>636</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
@@ -14308,7 +14465,7 @@
         <v>2699.97</v>
       </c>
       <c r="G5" s="58">
-        <f>F5-(E5*VLOOKUP(C5,$B$29:$F$38,5,FALSE))</f>
+        <f t="shared" ref="G5:G24" si="0">F5-(E5*VLOOKUP(C5,$B$29:$F$38,5,FALSE))</f>
         <v>839.9699999999998</v>
       </c>
     </row>
@@ -14329,7 +14486,7 @@
         <v>227.5</v>
       </c>
       <c r="G6" s="58">
-        <f t="shared" ref="G6:G24" si="0">F6-(E6*VLOOKUP(C6,$B$29:$F$38,5,FALSE))</f>
+        <f t="shared" si="0"/>
         <v>137.5</v>
       </c>
     </row>
@@ -14802,7 +14959,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" s="61" t="s">
         <v>591</v>
       </c>
@@ -14819,7 +14976,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" s="61" t="s">
         <v>596</v>
       </c>
@@ -14836,7 +14993,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B35" s="61" t="s">
         <v>601</v>
       </c>
@@ -14853,7 +15010,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B36" s="61" t="s">
         <v>606</v>
       </c>
@@ -14870,7 +15027,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B37" s="61" t="s">
         <v>613</v>
       </c>
@@ -14887,7 +15044,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38" s="61" t="s">
         <v>616</v>
       </c>
@@ -14904,79 +15061,8 @@
         <v>310</v>
       </c>
     </row>
-    <row r="42" spans="2:7" s="49" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="49" t="s">
-        <v>636</v>
-      </c>
-      <c r="G42" s="50"/>
-    </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B44" s="53" t="s">
-        <v>678</v>
-      </c>
-    </row>
-    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B45" s="53" t="s">
-        <v>679</v>
-      </c>
-    </row>
-    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B47" s="53" t="s">
-        <v>637</v>
-      </c>
-    </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B50" s="18" t="s">
-        <v>638</v>
-      </c>
-    </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B51" s="20"/>
-    </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B52" s="18" t="s">
-        <v>680</v>
-      </c>
-    </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B53" s="18" t="s">
-        <v>681</v>
-      </c>
-    </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B54" s="18" t="s">
-        <v>682</v>
-      </c>
-    </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B58" s="18" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B59" s="20"/>
-    </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B60" s="20" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B61" s="20" t="s">
-        <v>640</v>
-      </c>
-    </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B64" s="49" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B65" s="53" t="s">
-        <v>685</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>